<commit_message>
fistula XLSForms: drop duplicate yes_no choice list
KoboToolbox refused to deploy because rows 70-71 in the choices sheet
('yes_no' / 'yes' and 'yes_no' / 'no') duplicated rows 2-3. The yes_no
list is defined at the top of _common_choices already; the fistula
forms reuse it. Removed the redundant second definition.
</commit_message>
<xml_diff>
--- a/koboforms/KF-01_Client_Registration.xlsx
+++ b/koboforms/KF-01_Client_Registration.xlsx
@@ -1170,7 +1170,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D85"/>
+  <dimension ref="A1:D83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2608,44 +2608,44 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>yes_no</t>
+          <t>gender</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>02</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>হ্যাঁ</t>
+          <t>মহিলা</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>yes_no</t>
+          <t>gender</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>01</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>না</t>
+          <t>পুরুষ</t>
         </is>
       </c>
     </row>
@@ -2657,17 +2657,17 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>03</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Transgender</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>মহিলা</t>
+          <t>তৃতীয় লিঙ্গ</t>
         </is>
       </c>
     </row>
@@ -2679,61 +2679,61 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>04</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>পুরুষ</t>
+          <t>অন্যান্য</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>gender</t>
+          <t>target_group</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>05</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Transgender</t>
+          <t>FSW</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>তৃতীয় লিঙ্গ</t>
+          <t>এফএসডব্লিউ</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>gender</t>
+          <t>target_group</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>04</t>
+          <t>06</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>PWID</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>অন্যান্য</t>
+          <t>পিডব্লিউআইডি</t>
         </is>
       </c>
     </row>
@@ -2745,17 +2745,17 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>05</t>
+          <t>01</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>FSW</t>
+          <t>MSM</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>এফএসডব্লিউ</t>
+          <t>এমএসএম</t>
         </is>
       </c>
     </row>
@@ -2767,17 +2767,17 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>06</t>
+          <t>02</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>PWID</t>
+          <t>MSW / Kothi</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>পিডব্লিউআইডি</t>
+          <t>এমএসডব্লিউ / কথি</t>
         </is>
       </c>
     </row>
@@ -2789,17 +2789,17 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>03</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>MSM</t>
+          <t>Transgender</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>এমএসএম</t>
+          <t>তৃতীয় লিঙ্গ</t>
         </is>
       </c>
     </row>
@@ -2811,61 +2811,61 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>04</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>MSW / Kothi</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>এমএসডব্লিউ / কথি</t>
+          <t>অন্যান্য</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>target_group</t>
+          <t>survivor_gender</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>female</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Transgender</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>তৃতীয় লিঙ্গ</t>
+          <t>মহিলা</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>target_group</t>
+          <t>survivor_gender</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>04</t>
+          <t>male</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>Others</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>অন্যান্য</t>
+          <t>পুরুষ</t>
         </is>
       </c>
     </row>
@@ -2877,17 +2877,17 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>female</t>
+          <t>transgender</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Transgender</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>মহিলা</t>
+          <t>তৃতীয় লিঙ্গ</t>
         </is>
       </c>
     </row>
@@ -2899,59 +2899,15 @@
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>male</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
-        <is>
-          <t>পুরুষ</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="2" t="inlineStr">
-        <is>
-          <t>survivor_gender</t>
-        </is>
-      </c>
-      <c r="B84" s="2" t="inlineStr">
-        <is>
-          <t>transgender</t>
-        </is>
-      </c>
-      <c r="C84" s="2" t="inlineStr">
-        <is>
-          <t>Transgender</t>
-        </is>
-      </c>
-      <c r="D84" s="2" t="inlineStr">
-        <is>
-          <t>তৃতীয় লিঙ্গ</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="3" t="inlineStr">
-        <is>
-          <t>survivor_gender</t>
-        </is>
-      </c>
-      <c r="B85" s="3" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="C85" s="3" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="D85" s="3" t="inlineStr">
         <is>
           <t>অন্যান্য</t>
         </is>

</xml_diff>

<commit_message>
generate_kobo_forms: emit placeholder center_code when DB has none
XLSForm validators reject 'select_one center_code' fields whose
choices list is empty ("List name not in choices sheet: center_code").
Fistula forms hit this because the dev DB has no ServiceCenter rows
seeded for CIPRB.

_center_choices() now emits a single placeholder row when no active
centers exist, so the generated XLSForm always deploys. Replace with
real rows by seeding ServiceCenters and regenerating.
</commit_message>
<xml_diff>
--- a/koboforms/KF-01_Client_Registration.xlsx
+++ b/koboforms/KF-01_Client_Registration.xlsx
@@ -1170,7 +1170,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D83"/>
+  <dimension ref="A1:D84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2910,6 +2910,28 @@
       <c r="D83" s="3" t="inlineStr">
         <is>
           <t>অন্যান্য</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>center_code</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>PLACEHOLDER</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>Placeholder — seed ServiceCenters before deployment</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>প্লেসহোল্ডার — প্রকৃত কেন্দ্র যোগ করুন</t>
         </is>
       </c>
     </row>

</xml_diff>